<commit_message>
feat: BWCCI Fashion Design CS revised; mobile fixes
</commit_message>
<xml_diff>
--- a/data/xlsx/bwcci--fashion-design-product-development-and-entrepreneurship.xlsx
+++ b/data/xlsx/bwcci--fashion-design-product-development-and-entrepreneurship.xlsx
@@ -99,7 +99,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="bottom"/>
@@ -132,6 +132,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -497,7 +503,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G30"/>
+  <dimension ref="A1:G38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15.17" customWidth="1" min="1" max="1"/>
@@ -637,16 +643,16 @@
       </c>
     </row>
     <row r="16" ht="14.15" customHeight="1">
-      <c r="A16" s="7" t="n">
+      <c r="A16" s="14" t="n">
         <v>1</v>
       </c>
       <c r="B16" s="8" t="inlineStr">
         <is>
-          <t>Computers/Laptop</t>
+          <t>Computer / Laptop (with relevant design software)</t>
         </is>
       </c>
       <c r="C16" s="9" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D16" s="9" t="n"/>
       <c r="E16" s="9" t="n">
@@ -659,12 +665,12 @@
       <c r="G16" s="9" t="n"/>
     </row>
     <row r="17" ht="14.15" customHeight="1">
-      <c r="A17" s="7" t="n">
+      <c r="A17" s="14" t="n">
         <v>2</v>
       </c>
       <c r="B17" s="8" t="inlineStr">
         <is>
-          <t>Projector &amp; Screen (HD quality, HDMI support, 3000+ lumens)</t>
+          <t>Multimedia Projector &amp; Screen (HD quality, HDMI support)</t>
         </is>
       </c>
       <c r="C17" s="9" t="n">
@@ -681,7 +687,7 @@
       <c r="G17" s="9" t="n"/>
     </row>
     <row r="18" ht="14.15" customHeight="1">
-      <c r="A18" s="7" t="n">
+      <c r="A18" s="14" t="n">
         <v>3</v>
       </c>
       <c r="B18" s="8" t="inlineStr">
@@ -703,20 +709,20 @@
       <c r="G18" s="9" t="n"/>
     </row>
     <row r="19" ht="14.15" customHeight="1">
-      <c r="A19" s="7" t="n">
+      <c r="A19" s="14" t="n">
         <v>4</v>
       </c>
       <c r="B19" s="8" t="inlineStr">
         <is>
-          <t>Mannequins/Dress Forms (Female and male standard sizes)</t>
+          <t>Single Needle Lock Stitch Machine (Industrial/Domestic)</t>
         </is>
       </c>
       <c r="C19" s="9" t="n">
-        <v>2</v>
+        <v>25</v>
       </c>
       <c r="D19" s="9" t="n"/>
       <c r="E19" s="9" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F19" s="9">
         <f>IFERROR(MIN(C19,D19)*E19/C19,0)</f>
@@ -725,20 +731,20 @@
       <c r="G19" s="9" t="n"/>
     </row>
     <row r="20" ht="14.15" customHeight="1">
-      <c r="A20" s="7" t="n">
+      <c r="A20" s="14" t="n">
         <v>5</v>
       </c>
       <c r="B20" s="8" t="inlineStr">
         <is>
-          <t>Single needle lock stitch machine</t>
+          <t>Overlock Machine (3 or 4 threads)</t>
         </is>
       </c>
       <c r="C20" s="9" t="n">
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="D20" s="9" t="n"/>
       <c r="E20" s="9" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F20" s="9">
         <f>IFERROR(MIN(C20,D20)*E20/C20,0)</f>
@@ -747,20 +753,20 @@
       <c r="G20" s="9" t="n"/>
     </row>
     <row r="21" ht="14.15" customHeight="1">
-      <c r="A21" s="7" t="n">
+      <c r="A21" s="14" t="n">
         <v>6</v>
       </c>
       <c r="B21" s="8" t="inlineStr">
         <is>
-          <t>Overlock machine</t>
+          <t>Embroidery Machine (Manual/Computerized)</t>
         </is>
       </c>
       <c r="C21" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D21" s="9" t="n"/>
       <c r="E21" s="9" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="F21" s="9">
         <f>IFERROR(MIN(C21,D21)*E21/C21,0)</f>
@@ -769,20 +775,20 @@
       <c r="G21" s="9" t="n"/>
     </row>
     <row r="22" ht="14.15" customHeight="1">
-      <c r="A22" s="7" t="n">
+      <c r="A22" s="14" t="n">
         <v>7</v>
       </c>
       <c r="B22" s="8" t="inlineStr">
         <is>
-          <t>Cutting table (60”x 50”)</t>
+          <t>Button Hole Machine</t>
         </is>
       </c>
       <c r="C22" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D22" s="9" t="n"/>
       <c r="E22" s="9" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F22" s="9">
         <f>IFERROR(MIN(C22,D22)*E22/C22,0)</f>
@@ -791,12 +797,12 @@
       <c r="G22" s="9" t="n"/>
     </row>
     <row r="23" ht="14.15" customHeight="1">
-      <c r="A23" s="7" t="n">
+      <c r="A23" s="14" t="n">
         <v>8</v>
       </c>
       <c r="B23" s="8" t="inlineStr">
         <is>
-          <t>Electric iron</t>
+          <t>Button Stitch Machine</t>
         </is>
       </c>
       <c r="C23" s="9" t="n">
@@ -813,20 +819,20 @@
       <c r="G23" s="9" t="n"/>
     </row>
     <row r="24" ht="14.15" customHeight="1">
-      <c r="A24" s="7" t="n">
+      <c r="A24" s="14" t="n">
         <v>9</v>
       </c>
       <c r="B24" s="8" t="inlineStr">
         <is>
-          <t>Electric steam iron with iron table</t>
+          <t>Cutting Table (Standard size: min. 5ft - 60”x50”)</t>
         </is>
       </c>
       <c r="C24" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D24" s="9" t="n"/>
       <c r="E24" s="9" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F24" s="9">
         <f>IFERROR(MIN(C24,D24)*E24/C24,0)</f>
@@ -835,20 +841,20 @@
       <c r="G24" s="9" t="n"/>
     </row>
     <row r="25" ht="14.15" customHeight="1">
-      <c r="A25" s="7" t="n">
+      <c r="A25" s="14" t="n">
         <v>10</v>
       </c>
       <c r="B25" s="8" t="inlineStr">
         <is>
-          <t>Scissors (10”-12”)</t>
+          <t>Pattern Making &amp; Printing Table (Min 5ft)</t>
         </is>
       </c>
       <c r="C25" s="9" t="n">
-        <v>25</v>
+        <v>3</v>
       </c>
       <c r="D25" s="9" t="n"/>
       <c r="E25" s="9" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="F25" s="9">
         <f>IFERROR(MIN(C25,D25)*E25/C25,0)</f>
@@ -857,20 +863,20 @@
       <c r="G25" s="9" t="n"/>
     </row>
     <row r="26" ht="14.15" customHeight="1">
-      <c r="A26" s="7" t="n">
+      <c r="A26" s="14" t="n">
         <v>11</v>
       </c>
       <c r="B26" s="8" t="inlineStr">
         <is>
-          <t>Sewing tool box</t>
+          <t>Mannequins / Dress Forms (Male, Female, and Child standard sizes)</t>
         </is>
       </c>
       <c r="C26" s="9" t="n">
-        <v>25</v>
+        <v>5</v>
       </c>
       <c r="D26" s="9" t="n"/>
       <c r="E26" s="9" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="F26" s="9">
         <f>IFERROR(MIN(C26,D26)*E26/C26,0)</f>
@@ -878,57 +884,233 @@
       </c>
       <c r="G26" s="9" t="n"/>
     </row>
-    <row r="27">
-      <c r="A27" s="10" t="inlineStr">
+    <row r="27" ht="14.15" customHeight="1">
+      <c r="A27" s="14" t="n">
+        <v>12</v>
+      </c>
+      <c r="B27" s="8" t="inlineStr">
+        <is>
+          <t>Electric Steam Iron with Ironing Table</t>
+        </is>
+      </c>
+      <c r="C27" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="D27" s="9" t="n"/>
+      <c r="E27" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="F27" s="9">
+        <f>IFERROR(MIN(C27,D27)*E27/C27,0)</f>
+        <v/>
+      </c>
+      <c r="G27" s="9" t="n"/>
+    </row>
+    <row r="28" ht="14.15" customHeight="1">
+      <c r="A28" s="14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B28" s="8" t="inlineStr">
+        <is>
+          <t>Burner for Dyeing and Printing</t>
+        </is>
+      </c>
+      <c r="C28" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="D28" s="9" t="n"/>
+      <c r="E28" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="F28" s="9">
+        <f>IFERROR(MIN(C28,D28)*E28/C28,0)</f>
+        <v/>
+      </c>
+      <c r="G28" s="9" t="n"/>
+    </row>
+    <row r="29" ht="14.15" customHeight="1">
+      <c r="A29" s="14" t="n">
+        <v>14</v>
+      </c>
+      <c r="B29" s="8" t="inlineStr">
+        <is>
+          <t>Tracing Wheels</t>
+        </is>
+      </c>
+      <c r="C29" s="9" t="n">
+        <v>25</v>
+      </c>
+      <c r="D29" s="9" t="n"/>
+      <c r="E29" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="F29" s="9">
+        <f>IFERROR(MIN(C29,D29)*E29/C29,0)</f>
+        <v/>
+      </c>
+      <c r="G29" s="9" t="n"/>
+    </row>
+    <row r="30" ht="14.15" customHeight="1">
+      <c r="A30" s="14" t="n">
+        <v>15</v>
+      </c>
+      <c r="B30" s="8" t="inlineStr">
+        <is>
+          <t>Sets of Pattern Making Curves (French curve, Hip curve, etc.)</t>
+        </is>
+      </c>
+      <c r="C30" s="9" t="n">
+        <v>25</v>
+      </c>
+      <c r="D30" s="9" t="n"/>
+      <c r="E30" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="F30" s="9">
+        <f>IFERROR(MIN(C30,D30)*E30/C30,0)</f>
+        <v/>
+      </c>
+      <c r="G30" s="9" t="n"/>
+    </row>
+    <row r="31" ht="14.15" customHeight="1">
+      <c r="A31" s="14" t="n">
+        <v>16</v>
+      </c>
+      <c r="B31" s="8" t="inlineStr">
+        <is>
+          <t>Fabric Cutting Scissors (10”-12”)</t>
+        </is>
+      </c>
+      <c r="C31" s="9" t="n">
+        <v>25</v>
+      </c>
+      <c r="D31" s="9" t="n"/>
+      <c r="E31" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="F31" s="9">
+        <f>IFERROR(MIN(C31,D31)*E31/C31,0)</f>
+        <v/>
+      </c>
+      <c r="G31" s="9" t="n"/>
+    </row>
+    <row r="32" ht="14.15" customHeight="1">
+      <c r="A32" s="14" t="n">
+        <v>17</v>
+      </c>
+      <c r="B32" s="8" t="inlineStr">
+        <is>
+          <t>Different Screen for Printing</t>
+        </is>
+      </c>
+      <c r="C32" s="9" t="n">
+        <v>10</v>
+      </c>
+      <c r="D32" s="9" t="n"/>
+      <c r="E32" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="F32" s="9">
+        <f>IFERROR(MIN(C32,D32)*E32/C32,0)</f>
+        <v/>
+      </c>
+      <c r="G32" s="9" t="n"/>
+    </row>
+    <row r="33" ht="14.15" customHeight="1">
+      <c r="A33" s="14" t="n">
+        <v>18</v>
+      </c>
+      <c r="B33" s="8" t="inlineStr">
+        <is>
+          <t>Different Dices for Block Printing</t>
+        </is>
+      </c>
+      <c r="C33" s="9" t="n">
+        <v>15</v>
+      </c>
+      <c r="D33" s="9" t="n"/>
+      <c r="E33" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="F33" s="9">
+        <f>IFERROR(MIN(C33,D33)*E33/C33,0)</f>
+        <v/>
+      </c>
+      <c r="G33" s="9" t="n"/>
+    </row>
+    <row r="34" ht="14.15" customHeight="1">
+      <c r="A34" s="14" t="n">
+        <v>19</v>
+      </c>
+      <c r="B34" s="8" t="inlineStr">
+        <is>
+          <t>Sewing Tool Box (Measuring tape, tailor’s chalk, needles, etc.)</t>
+        </is>
+      </c>
+      <c r="C34" s="9" t="n">
+        <v>25</v>
+      </c>
+      <c r="D34" s="9" t="n"/>
+      <c r="E34" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="F34" s="9">
+        <f>IFERROR(MIN(C34,D34)*E34/C34,0)</f>
+        <v/>
+      </c>
+      <c r="G34" s="9" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="15" t="inlineStr">
         <is>
           <t>Sum</t>
         </is>
       </c>
-      <c r="B27" s="11" t="n"/>
-      <c r="C27" s="11" t="n"/>
-      <c r="D27" s="12" t="n"/>
-      <c r="E27" s="10">
-        <f>SUM(E16:E26)</f>
-        <v/>
-      </c>
-      <c r="F27" s="10">
-        <f>SUM(F16:F26)</f>
-        <v/>
-      </c>
-      <c r="G27" s="13" t="n"/>
-    </row>
-    <row r="28">
-      <c r="A28" s="10" t="inlineStr">
+      <c r="B35" s="11" t="n"/>
+      <c r="C35" s="11" t="n"/>
+      <c r="D35" s="12" t="n"/>
+      <c r="E35" s="15">
+        <f>SUM(E16:E34)</f>
+        <v/>
+      </c>
+      <c r="F35" s="15">
+        <f>SUM(F16:F34)</f>
+        <v/>
+      </c>
+      <c r="G35" s="13" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="15" t="inlineStr">
         <is>
           <t>Score out of 100</t>
         </is>
       </c>
-      <c r="B28" s="11" t="n"/>
-      <c r="C28" s="11" t="n"/>
-      <c r="D28" s="11" t="n"/>
-      <c r="E28" s="12" t="n"/>
-      <c r="F28" s="10">
-        <f>F27/E27*100</f>
-        <v/>
-      </c>
-      <c r="G28" s="13" t="n"/>
-    </row>
-    <row r="29" ht="9.75" customHeight="1"/>
-    <row r="30">
-      <c r="A30" s="10" t="inlineStr">
+      <c r="B36" s="11" t="n"/>
+      <c r="C36" s="11" t="n"/>
+      <c r="D36" s="11" t="n"/>
+      <c r="E36" s="12" t="n"/>
+      <c r="F36" s="15">
+        <f>F35/E35*100</f>
+        <v/>
+      </c>
+      <c r="G36" s="13" t="n"/>
+    </row>
+    <row r="37" ht="9.75" customHeight="1"/>
+    <row r="38">
+      <c r="A38" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">Total achieved points out of 30  </t>
         </is>
       </c>
-      <c r="B30" s="11" t="n"/>
-      <c r="C30" s="11" t="n"/>
-      <c r="D30" s="11" t="n"/>
-      <c r="E30" s="12" t="n"/>
-      <c r="F30" s="10">
-        <f>F28*30/100</f>
-        <v/>
-      </c>
-      <c r="G30" s="10" t="inlineStr">
+      <c r="B38" s="11" t="n"/>
+      <c r="C38" s="11" t="n"/>
+      <c r="D38" s="11" t="n"/>
+      <c r="E38" s="12" t="n"/>
+      <c r="F38" s="15">
+        <f>F36*30/100</f>
+        <v/>
+      </c>
+      <c r="G38" s="15" t="inlineStr">
         <is>
           <t>Points</t>
         </is>
@@ -936,14 +1118,14 @@
     </row>
   </sheetData>
   <mergeCells count="8">
-    <mergeCell ref="A30:E30"/>
     <mergeCell ref="A13:G13"/>
     <mergeCell ref="C7:G7"/>
-    <mergeCell ref="A27:D27"/>
     <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A28:E28"/>
-    <mergeCell ref="A29:G29"/>
+    <mergeCell ref="A38:E38"/>
+    <mergeCell ref="A35:D35"/>
+    <mergeCell ref="A36:E36"/>
     <mergeCell ref="C8:G8"/>
+    <mergeCell ref="A37:G37"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>